<commit_message>
feat: perbarui benchmark 14 skenario AES vs ChaCha20 dan sesuaikan eksportir Excel 10 kolom
</commit_message>
<xml_diff>
--- a/docs/hasil_pengujian_kriptografi.xlsx
+++ b/docs/hasil_pengujian_kriptografi.xlsx
@@ -164,30 +164,6 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Hasil Pengujian'!C1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Hasil Pengujian'!$A$2:$A$11</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Hasil Pengujian'!$C$2:$C$11</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
               <f>'Hasil Pengujian'!D1</f>
             </strRef>
           </tx>
@@ -198,12 +174,36 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Hasil Pengujian'!$A$2:$A$11</f>
+              <f>'Hasil Pengujian'!$A$2:$A$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Hasil Pengujian'!$D$2:$D$11</f>
+              <f>'Hasil Pengujian'!$D$2:$D$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Hasil Pengujian'!E1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Hasil Pengujian'!$A$2:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Hasil Pengujian'!$E$2:$E$15</f>
             </numRef>
           </val>
         </ser>
@@ -277,7 +277,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>9</col>
+      <col>11</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -589,56 +589,68 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="63" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="63" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Nama Berkas / Skenario</t>
+          <t>Nama Berkas</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Ukuran (Bytes)</t>
+          <t>Algoritma</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Ukuran (byte)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Waktu Enkripsi (ms)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Waktu Dekripsi (ms)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Entropi Plaintext</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Entropi Ciphertext</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Avalanche Effect (%)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Dekripsi Identik</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Keterangan</t>
         </is>
@@ -647,28 +659,38 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>File Teks (1 KB)</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+          <t>File Teks 1 KB</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AES-256-GCM</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>1048</v>
       </c>
-      <c r="C2" t="n">
-        <v>515.9</v>
-      </c>
       <c r="D2" t="n">
-        <v>574.59</v>
+        <v>528.6</v>
       </c>
       <c r="E2" t="n">
+        <v>576.5</v>
+      </c>
+      <c r="F2" t="n">
         <v>4.9467</v>
       </c>
-      <c r="F2" t="n">
-        <v>7.8053</v>
-      </c>
       <c r="G2" t="n">
-        <v>49.62</v>
-      </c>
-      <c r="H2" t="inlineStr">
+        <v>7.8198</v>
+      </c>
+      <c r="H2" t="n">
+        <v>50.32</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>Entropi tinggi - ciphertext tampak acak</t>
         </is>
@@ -677,58 +699,78 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>File Teks (100 KB)</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>4100</v>
+          <t>File Teks 1 KB</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ChaCha20-Poly1305</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>494.2</v>
+        <v>1048</v>
       </c>
       <c r="D3" t="n">
-        <v>560.41</v>
+        <v>485</v>
       </c>
       <c r="E3" t="n">
-        <v>4.0162</v>
+        <v>507.8</v>
       </c>
       <c r="F3" t="n">
-        <v>7.9527</v>
+        <v>4.9467</v>
       </c>
       <c r="G3" t="n">
-        <v>50.08</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Entropi mendekati maksimum (8.0) - ciphertext acak sempurna</t>
+        <v>7.7859</v>
+      </c>
+      <c r="H3" t="n">
+        <v>49.92</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Entropi tinggi - ciphertext tampak acak</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>File Teks (1 MB)</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+          <t>File Teks 1 MB</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AES-256-GCM</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>1048576</v>
       </c>
-      <c r="C4" t="n">
-        <v>507.2</v>
-      </c>
       <c r="D4" t="n">
-        <v>544.85</v>
+        <v>477.81</v>
       </c>
       <c r="E4" t="n">
+        <v>500.03</v>
+      </c>
+      <c r="F4" t="n">
         <v>4.8803</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>7.9998</v>
       </c>
-      <c r="G4" t="n">
-        <v>50.01</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" t="n">
+        <v>49.98</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>Entropi mendekati maksimum (8.0) - ciphertext acak sempurna</t>
         </is>
@@ -737,28 +779,38 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>File Teks (10 MB)</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>10485760</v>
+          <t>File Teks 1 MB</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ChaCha20-Poly1305</t>
+        </is>
       </c>
       <c r="C5" t="n">
-        <v>557.09</v>
+        <v>1048576</v>
       </c>
       <c r="D5" t="n">
-        <v>524.91</v>
+        <v>508.95</v>
       </c>
       <c r="E5" t="n">
+        <v>498.9</v>
+      </c>
+      <c r="F5" t="n">
         <v>4.8803</v>
       </c>
-      <c r="F5" t="n">
-        <v>8</v>
-      </c>
       <c r="G5" t="n">
-        <v>49.99</v>
-      </c>
-      <c r="H5" t="inlineStr">
+        <v>7.9998</v>
+      </c>
+      <c r="H5" t="n">
+        <v>50</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Entropi mendekati maksimum (8.0) - ciphertext acak sempurna</t>
         </is>
@@ -767,58 +819,78 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>File PDF</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1070</v>
+          <t>File Teks 10 MB</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AES-256-GCM</t>
+        </is>
       </c>
       <c r="C6" t="n">
-        <v>508.73</v>
+        <v>10485760</v>
       </c>
       <c r="D6" t="n">
-        <v>479.85</v>
+        <v>584.59</v>
       </c>
       <c r="E6" t="n">
-        <v>5.7621</v>
+        <v>525.04</v>
       </c>
       <c r="F6" t="n">
-        <v>7.8095</v>
+        <v>4.8803</v>
       </c>
       <c r="G6" t="n">
-        <v>50.07</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Entropi tinggi - ciphertext tampak acak</t>
+        <v>8</v>
+      </c>
+      <c r="H6" t="n">
+        <v>50</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Entropi mendekati maksimum (8.0) - ciphertext acak sempurna</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gambar Uncompressed BMP</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>120054</v>
+          <t>File Teks 10 MB</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ChaCha20-Poly1305</t>
+        </is>
       </c>
       <c r="C7" t="n">
-        <v>483.9</v>
+        <v>10485760</v>
       </c>
       <c r="D7" t="n">
-        <v>484.14</v>
+        <v>613.54</v>
       </c>
       <c r="E7" t="n">
-        <v>0.7823</v>
+        <v>627.53</v>
       </c>
       <c r="F7" t="n">
-        <v>7.9984</v>
+        <v>4.8803</v>
       </c>
       <c r="G7" t="n">
-        <v>49.9</v>
-      </c>
-      <c r="H7" t="inlineStr">
+        <v>8</v>
+      </c>
+      <c r="H7" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>Entropi mendekati maksimum (8.0) - ciphertext acak sempurna</t>
         </is>
@@ -827,28 +899,38 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Gambar Compressed PNG</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>862</v>
+          <t>Dokumen PDF</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>AES-256-GCM</t>
+        </is>
       </c>
       <c r="C8" t="n">
-        <v>533.97</v>
+        <v>1070</v>
       </c>
       <c r="D8" t="n">
-        <v>480.87</v>
+        <v>495.43</v>
       </c>
       <c r="E8" t="n">
-        <v>6.6672</v>
+        <v>496.04</v>
       </c>
       <c r="F8" t="n">
-        <v>7.7789</v>
+        <v>5.7621</v>
       </c>
       <c r="G8" t="n">
-        <v>50.23</v>
-      </c>
-      <c r="H8" t="inlineStr">
+        <v>7.7999</v>
+      </c>
+      <c r="H8" t="n">
+        <v>48.97</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>Entropi tinggi - ciphertext tampak acak</t>
         </is>
@@ -857,90 +939,280 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>File Struktur Data JSON</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>4100</v>
+          <t>Dokumen PDF</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ChaCha20-Poly1305</t>
+        </is>
       </c>
       <c r="C9" t="n">
-        <v>485.15</v>
+        <v>1070</v>
       </c>
       <c r="D9" t="n">
-        <v>477.32</v>
+        <v>500.68</v>
       </c>
       <c r="E9" t="n">
-        <v>4.0162</v>
+        <v>499.09</v>
       </c>
       <c r="F9" t="n">
-        <v>7.9491</v>
+        <v>5.7621</v>
       </c>
       <c r="G9" t="n">
-        <v>50.16</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Entropi mendekati maksimum (8.0) - ciphertext acak sempurna</t>
+        <v>7.7959</v>
+      </c>
+      <c r="H9" t="n">
+        <v>50.43</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Entropi tinggi - ciphertext tampak acak</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Simulasi Cipherteks Rusak (1-Byte Corrupt)</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1070</v>
+          <t>Gambar BMP</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>AES-256-GCM</t>
+        </is>
       </c>
       <c r="C10" t="n">
-        <v>485.78</v>
+        <v>120054</v>
       </c>
       <c r="D10" t="n">
-        <v>490.06</v>
+        <v>506.09</v>
       </c>
       <c r="E10" t="n">
-        <v>5.7621</v>
+        <v>480.97</v>
       </c>
       <c r="F10" t="n">
-        <v>7.7827</v>
+        <v>0.7823</v>
       </c>
       <c r="G10" t="n">
-        <v>49.74</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Entropi tinggi - ciphertext tampak acak</t>
+        <v>7.9987</v>
+      </c>
+      <c r="H10" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Entropi mendekati maksimum (8.0) - ciphertext acak sempurna</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Simulasi Bit-Flip Kunci (Avalanche Test)</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>1048576</v>
+          <t>Gambar BMP</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ChaCha20-Poly1305</t>
+        </is>
       </c>
       <c r="C11" t="n">
-        <v>489.1</v>
+        <v>120054</v>
       </c>
       <c r="D11" t="n">
-        <v>604.14</v>
+        <v>494.36</v>
       </c>
       <c r="E11" t="n">
-        <v>4.8803</v>
+        <v>496.22</v>
       </c>
       <c r="F11" t="n">
-        <v>7.9998</v>
+        <v>0.7823</v>
       </c>
       <c r="G11" t="n">
-        <v>49.99</v>
-      </c>
-      <c r="H11" t="inlineStr">
+        <v>7.9988</v>
+      </c>
+      <c r="H11" t="n">
+        <v>50.07</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
         <is>
           <t>Entropi mendekati maksimum (8.0) - ciphertext acak sempurna</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Gambar JPG</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>AES-256-GCM</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2893</v>
+      </c>
+      <c r="D12" t="n">
+        <v>479.8</v>
+      </c>
+      <c r="E12" t="n">
+        <v>542.8</v>
+      </c>
+      <c r="F12" t="n">
+        <v>7.3027</v>
+      </c>
+      <c r="G12" t="n">
+        <v>7.931</v>
+      </c>
+      <c r="H12" t="n">
+        <v>49.87</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Entropi mendekati maksimum (8.0) - ciphertext acak sempurna</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Gambar JPG</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ChaCha20-Poly1305</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2893</v>
+      </c>
+      <c r="D13" t="n">
+        <v>483.07</v>
+      </c>
+      <c r="E13" t="n">
+        <v>476.08</v>
+      </c>
+      <c r="F13" t="n">
+        <v>7.3027</v>
+      </c>
+      <c r="G13" t="n">
+        <v>7.9351</v>
+      </c>
+      <c r="H13" t="n">
+        <v>50</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Entropi mendekati maksimum (8.0) - ciphertext acak sempurna</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Gambar PNG</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>AES-256-GCM</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>862</v>
+      </c>
+      <c r="D14" t="n">
+        <v>480.57</v>
+      </c>
+      <c r="E14" t="n">
+        <v>481.45</v>
+      </c>
+      <c r="F14" t="n">
+        <v>6.6672</v>
+      </c>
+      <c r="G14" t="n">
+        <v>7.7579</v>
+      </c>
+      <c r="H14" t="n">
+        <v>49.22</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Entropi tinggi - ciphertext tampak acak</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Gambar PNG</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ChaCha20-Poly1305</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>862</v>
+      </c>
+      <c r="D15" t="n">
+        <v>492.56</v>
+      </c>
+      <c r="E15" t="n">
+        <v>497.42</v>
+      </c>
+      <c r="F15" t="n">
+        <v>6.6672</v>
+      </c>
+      <c r="G15" t="n">
+        <v>7.7917</v>
+      </c>
+      <c r="H15" t="n">
+        <v>50.84</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Entropi tinggi - ciphertext tampak acak</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: commit file uji asli (PDF/BMP/JPG/PNG) yang sebelumnya cuma ada lokal, supaya hasil bisa direproduksi dari repo
</commit_message>
<xml_diff>
--- a/docs/hasil_pengujian_kriptografi.xlsx
+++ b/docs/hasil_pengujian_kriptografi.xlsx
@@ -668,22 +668,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1048</v>
+        <v>1024</v>
       </c>
       <c r="D2" t="n">
-        <v>528.6</v>
+        <v>594.49</v>
       </c>
       <c r="E2" t="n">
-        <v>576.5</v>
+        <v>629.5599999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>4.9467</v>
+        <v>4.8781</v>
       </c>
       <c r="G2" t="n">
-        <v>7.8198</v>
+        <v>7.8168</v>
       </c>
       <c r="H2" t="n">
-        <v>50.32</v>
+        <v>50.7</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -708,22 +708,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1048</v>
+        <v>1024</v>
       </c>
       <c r="D3" t="n">
-        <v>485</v>
+        <v>493.51</v>
       </c>
       <c r="E3" t="n">
-        <v>507.8</v>
+        <v>495.9</v>
       </c>
       <c r="F3" t="n">
-        <v>4.9467</v>
+        <v>4.8781</v>
       </c>
       <c r="G3" t="n">
-        <v>7.7859</v>
+        <v>7.8054</v>
       </c>
       <c r="H3" t="n">
-        <v>49.92</v>
+        <v>49.82</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -751,10 +751,10 @@
         <v>1048576</v>
       </c>
       <c r="D4" t="n">
-        <v>477.81</v>
+        <v>501.41</v>
       </c>
       <c r="E4" t="n">
-        <v>500.03</v>
+        <v>520.22</v>
       </c>
       <c r="F4" t="n">
         <v>4.8803</v>
@@ -763,7 +763,7 @@
         <v>7.9998</v>
       </c>
       <c r="H4" t="n">
-        <v>49.98</v>
+        <v>50.05</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -791,19 +791,19 @@
         <v>1048576</v>
       </c>
       <c r="D5" t="n">
-        <v>508.95</v>
+        <v>512.48</v>
       </c>
       <c r="E5" t="n">
-        <v>498.9</v>
+        <v>490.57</v>
       </c>
       <c r="F5" t="n">
         <v>4.8803</v>
       </c>
       <c r="G5" t="n">
-        <v>7.9998</v>
+        <v>7.9999</v>
       </c>
       <c r="H5" t="n">
-        <v>50</v>
+        <v>49.99</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -831,10 +831,10 @@
         <v>10485760</v>
       </c>
       <c r="D6" t="n">
-        <v>584.59</v>
+        <v>556.1</v>
       </c>
       <c r="E6" t="n">
-        <v>525.04</v>
+        <v>534.51</v>
       </c>
       <c r="F6" t="n">
         <v>4.8803</v>
@@ -871,10 +871,10 @@
         <v>10485760</v>
       </c>
       <c r="D7" t="n">
-        <v>613.54</v>
+        <v>612.25</v>
       </c>
       <c r="E7" t="n">
-        <v>627.53</v>
+        <v>582.8099999999999</v>
       </c>
       <c r="F7" t="n">
         <v>4.8803</v>
@@ -883,7 +883,7 @@
         <v>8</v>
       </c>
       <c r="H7" t="n">
-        <v>49.99</v>
+        <v>50</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -908,22 +908,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1070</v>
+        <v>12303288</v>
       </c>
       <c r="D8" t="n">
-        <v>495.43</v>
+        <v>566.83</v>
       </c>
       <c r="E8" t="n">
-        <v>496.04</v>
+        <v>579.38</v>
       </c>
       <c r="F8" t="n">
-        <v>5.7621</v>
+        <v>7.9943</v>
       </c>
       <c r="G8" t="n">
-        <v>7.7999</v>
+        <v>8</v>
       </c>
       <c r="H8" t="n">
-        <v>48.97</v>
+        <v>50</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -932,7 +932,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Entropi tinggi - ciphertext tampak acak</t>
+          <t>Entropi mendekati maksimum (8.0) - ciphertext acak sempurna</t>
         </is>
       </c>
     </row>
@@ -948,22 +948,22 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1070</v>
+        <v>12303288</v>
       </c>
       <c r="D9" t="n">
-        <v>500.68</v>
+        <v>682.95</v>
       </c>
       <c r="E9" t="n">
-        <v>499.09</v>
+        <v>662.64</v>
       </c>
       <c r="F9" t="n">
-        <v>5.7621</v>
+        <v>7.9943</v>
       </c>
       <c r="G9" t="n">
-        <v>7.7959</v>
+        <v>8</v>
       </c>
       <c r="H9" t="n">
-        <v>50.43</v>
+        <v>50.01</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -972,7 +972,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Entropi tinggi - ciphertext tampak acak</t>
+          <t>Entropi mendekati maksimum (8.0) - ciphertext acak sempurna</t>
         </is>
       </c>
     </row>
@@ -988,22 +988,22 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>120054</v>
+        <v>6635574</v>
       </c>
       <c r="D10" t="n">
-        <v>506.09</v>
+        <v>557.51</v>
       </c>
       <c r="E10" t="n">
-        <v>480.97</v>
+        <v>530.11</v>
       </c>
       <c r="F10" t="n">
-        <v>0.7823</v>
+        <v>6.6398</v>
       </c>
       <c r="G10" t="n">
-        <v>7.9987</v>
+        <v>8</v>
       </c>
       <c r="H10" t="n">
-        <v>49.88</v>
+        <v>50</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1028,22 +1028,22 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>120054</v>
+        <v>6635574</v>
       </c>
       <c r="D11" t="n">
-        <v>494.36</v>
+        <v>552.25</v>
       </c>
       <c r="E11" t="n">
-        <v>496.22</v>
+        <v>549.53</v>
       </c>
       <c r="F11" t="n">
-        <v>0.7823</v>
+        <v>6.6398</v>
       </c>
       <c r="G11" t="n">
-        <v>7.9988</v>
+        <v>8</v>
       </c>
       <c r="H11" t="n">
-        <v>50.07</v>
+        <v>50</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1068,22 +1068,22 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2893</v>
+        <v>107357</v>
       </c>
       <c r="D12" t="n">
-        <v>479.8</v>
+        <v>505.4</v>
       </c>
       <c r="E12" t="n">
-        <v>542.8</v>
+        <v>583.23</v>
       </c>
       <c r="F12" t="n">
-        <v>7.3027</v>
+        <v>7.5312</v>
       </c>
       <c r="G12" t="n">
-        <v>7.931</v>
+        <v>7.9982</v>
       </c>
       <c r="H12" t="n">
-        <v>49.87</v>
+        <v>50.01</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1108,22 +1108,22 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2893</v>
+        <v>107357</v>
       </c>
       <c r="D13" t="n">
-        <v>483.07</v>
+        <v>505.55</v>
       </c>
       <c r="E13" t="n">
-        <v>476.08</v>
+        <v>502.55</v>
       </c>
       <c r="F13" t="n">
-        <v>7.3027</v>
+        <v>7.5312</v>
       </c>
       <c r="G13" t="n">
-        <v>7.9351</v>
+        <v>7.9983</v>
       </c>
       <c r="H13" t="n">
-        <v>50</v>
+        <v>49.99</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1148,22 +1148,22 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>862</v>
+        <v>1400325</v>
       </c>
       <c r="D14" t="n">
-        <v>480.57</v>
+        <v>513.77</v>
       </c>
       <c r="E14" t="n">
-        <v>481.45</v>
+        <v>518.92</v>
       </c>
       <c r="F14" t="n">
-        <v>6.6672</v>
+        <v>7.9882</v>
       </c>
       <c r="G14" t="n">
-        <v>7.7579</v>
+        <v>7.9999</v>
       </c>
       <c r="H14" t="n">
-        <v>49.22</v>
+        <v>49.99</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Entropi tinggi - ciphertext tampak acak</t>
+          <t>Entropi mendekati maksimum (8.0) - ciphertext acak sempurna</t>
         </is>
       </c>
     </row>
@@ -1188,22 +1188,22 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>862</v>
+        <v>1400325</v>
       </c>
       <c r="D15" t="n">
-        <v>492.56</v>
+        <v>512.41</v>
       </c>
       <c r="E15" t="n">
-        <v>497.42</v>
+        <v>500.19</v>
       </c>
       <c r="F15" t="n">
-        <v>6.6672</v>
+        <v>7.9882</v>
       </c>
       <c r="G15" t="n">
-        <v>7.7917</v>
+        <v>7.9999</v>
       </c>
       <c r="H15" t="n">
-        <v>50.84</v>
+        <v>49.99</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Entropi tinggi - ciphertext tampak acak</t>
+          <t>Entropi mendekati maksimum (8.0) - ciphertext acak sempurna</t>
         </is>
       </c>
     </row>

</xml_diff>